<commit_message>
add Week 11_LabX BASIC
</commit_message>
<xml_diff>
--- a/Sec2_Week10_LabX ADV_663380518_4/data/output_report.xlsx
+++ b/Sec2_Week10_LabX ADV_663380518_4/data/output_report.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <bookViews>
-    <workbookView activeTab="2"/>
+    <workbookView firstSheet="2" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" name="Audit Log" sheetId="1"/>
@@ -1459,7 +1459,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{BBE14E24-14E7-475D-B6D6-750706970DD4}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{AED28619-E21A-4CDE-8DEB-269FEEB650D2}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
@@ -1619,7 +1619,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{86C37668-9624-4C31-945B-B97FB1A33E76}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{5FB9F968-B7BE-4D10-AE49-04F079E8E249}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
@@ -1746,7 +1746,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{CC1CD556-C8AA-4A22-8B92-1F4D8436A2C1}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{7B65CB72-9F30-403C-8C8D-913385190078}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:O100"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>

</xml_diff>